<commit_message>
docs: replace proposal pptx with PDF, add Gantt chart PDF, and update schedule
</commit_message>
<xml_diff>
--- a/docs/PrivaLens_Gantt_Chart.xlsx
+++ b/docs/PrivaLens_Gantt_Chart.xlsx
@@ -1166,7 +1166,7 @@
         </is>
       </c>
       <c r="E3" s="81" t="n">
-        <v>46274</v>
+        <v>46281</v>
       </c>
       <c r="F3" s="82" t="n"/>
     </row>
@@ -2878,7 +2878,7 @@
         </is>
       </c>
       <c r="D21" s="36" t="n">
-        <v>0.5</v>
+        <v>0.85</v>
       </c>
       <c r="E21" s="37" t="n">
         <v>46272</v>
@@ -2961,7 +2961,7 @@
         </is>
       </c>
       <c r="D22" s="36" t="n">
-        <v>0.25</v>
+        <v>0.35</v>
       </c>
       <c r="E22" s="37" t="n">
         <v>46279</v>
@@ -3044,7 +3044,7 @@
         </is>
       </c>
       <c r="D23" s="36" t="n">
-        <v>0.4</v>
+        <v>0.55</v>
       </c>
       <c r="E23" s="37" t="n">
         <v>46277</v>
@@ -3127,7 +3127,7 @@
         </is>
       </c>
       <c r="D24" s="36" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="E24" s="37" t="n">
         <v>46274</v>
@@ -3210,7 +3210,7 @@
         </is>
       </c>
       <c r="D25" s="36" t="n">
-        <v>0.5</v>
+        <v>0.65</v>
       </c>
       <c r="E25" s="37" t="n">
         <v>46291</v>

</xml_diff>

<commit_message>
docs: add UML Class & Sequence Diagrams by Naman Arora, update Gantt chart, journals, and project structure
</commit_message>
<xml_diff>
--- a/docs/PrivaLens_Gantt_Chart.xlsx
+++ b/docs/PrivaLens_Gantt_Chart.xlsx
@@ -1166,7 +1166,7 @@
         </is>
       </c>
       <c r="E3" s="81" t="n">
-        <v>46281</v>
+        <v>46312</v>
       </c>
       <c r="F3" s="82" t="n"/>
     </row>
@@ -1177,7 +1177,7 @@
         </is>
       </c>
       <c r="E4" s="4" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="I4" s="75">
         <f>I5</f>
@@ -2878,7 +2878,7 @@
         </is>
       </c>
       <c r="D21" s="36" t="n">
-        <v>0.85</v>
+        <v>1</v>
       </c>
       <c r="E21" s="37" t="n">
         <v>46272</v>
@@ -2961,7 +2961,7 @@
         </is>
       </c>
       <c r="D22" s="36" t="n">
-        <v>0.35</v>
+        <v>1</v>
       </c>
       <c r="E22" s="37" t="n">
         <v>46279</v>
@@ -3044,7 +3044,7 @@
         </is>
       </c>
       <c r="D23" s="36" t="n">
-        <v>0.55</v>
+        <v>1</v>
       </c>
       <c r="E23" s="37" t="n">
         <v>46277</v>
@@ -3127,7 +3127,7 @@
         </is>
       </c>
       <c r="D24" s="36" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E24" s="37" t="n">
         <v>46274</v>
@@ -3210,7 +3210,7 @@
         </is>
       </c>
       <c r="D25" s="36" t="n">
-        <v>0.65</v>
+        <v>1</v>
       </c>
       <c r="E25" s="37" t="n">
         <v>46291</v>
@@ -3366,7 +3366,7 @@
         </is>
       </c>
       <c r="D27" s="42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E27" s="43" t="n">
         <v>46300</v>
@@ -3449,7 +3449,7 @@
         </is>
       </c>
       <c r="D28" s="42" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="E28" s="43" t="n">
         <v>46304</v>
@@ -3532,7 +3532,7 @@
         </is>
       </c>
       <c r="D29" s="42" t="n">
-        <v>0</v>
+        <v>0.85</v>
       </c>
       <c r="E29" s="43" t="n">
         <v>46307</v>
@@ -3615,7 +3615,7 @@
         </is>
       </c>
       <c r="D30" s="42" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="E30" s="43" t="n">
         <v>46311</v>
@@ -3698,7 +3698,7 @@
         </is>
       </c>
       <c r="D31" s="42" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="E31" s="43" t="n">
         <v>46313</v>

</xml_diff>